<commit_message>
Add cost columns to Full Results and a short walkthrough script
step1-4_summary.xlsx: Full Results now shows prompt_tokens,
completion_tokens, total_tokens, and latency_seconds per row, plus a
summary line with total cost, per-run average, and the three most
expensive runs.

evaluations/WALKTHROUGH_SCRIPT_2026-09-06.md: a tighter ~2-3 minute script
covering what changed, what improved, what still fails, and what's next.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/evaluations/step1-4_summary.xlsx
+++ b/evaluations/step1-4_summary.xlsx
@@ -2245,7 +2245,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G43"/>
+  <dimension ref="A1:K44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2254,7 +2254,11 @@
     <col width="30" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="55" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="55" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2304,6 +2308,26 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
+          <t>prompt_tokens</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>completion_tokens</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>total_tokens</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>latency_seconds</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
           <t>failure_category (participant-assigned)</t>
         </is>
       </c>
@@ -2337,7 +2361,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="3" t="n">
+        <v>32466</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>2581</v>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>35047</v>
+      </c>
+      <c r="J4" s="3" t="n">
+        <v>27.47</v>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -2372,7 +2408,19 @@
           <t>FAIL</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="G5" s="3" t="n">
+        <v>32224</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>4747</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>36971</v>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v>45.34</v>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
         <is>
           <t>Premature mutation proposal (not yet fixed)</t>
         </is>
@@ -2407,7 +2455,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="G6" s="3" t="n">
+        <v>21291</v>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>1110</v>
+      </c>
+      <c r="I6" s="3" t="n">
+        <v>22401</v>
+      </c>
+      <c r="J6" s="3" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="K6" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -2442,7 +2502,19 @@
           <t>FAIL</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="G7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="3" t="n">
+        <v>60.04</v>
+      </c>
+      <c r="K7" s="3" t="inlineStr">
         <is>
           <t>Provider/model latency instability</t>
         </is>
@@ -2477,6 +2549,26 @@
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="inlineStr">
+        <is>
           <t>N/A - fixture not yet implemented</t>
         </is>
       </c>
@@ -2510,7 +2602,19 @@
           <t>FAIL</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="G9" s="3" t="n">
+        <v>10586</v>
+      </c>
+      <c r="H9" s="3" t="n">
+        <v>2666</v>
+      </c>
+      <c r="I9" s="3" t="n">
+        <v>13252</v>
+      </c>
+      <c r="J9" s="3" t="n">
+        <v>13.86</v>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
         <is>
           <t>Under-specified relative time (Fix 2 pattern) - PARTIALLY FIXED 2026-09-06 (this row predates the fix). After the fix, shown 4 different behaviors across verification runs: resolves via list_events and reasons manually (no check_conflicts call), two runtime_error/timeout results, and one run that erroneously delegates via task instead of staying fast-path. Improved but not reliably fixed; see Step 2/4, Fix 7.</t>
         </is>
@@ -2545,7 +2649,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="G10" s="3" t="inlineStr">
+      <c r="G10" s="3" t="n">
+        <v>32941</v>
+      </c>
+      <c r="H10" s="3" t="n">
+        <v>2017</v>
+      </c>
+      <c r="I10" s="3" t="n">
+        <v>34958</v>
+      </c>
+      <c r="J10" s="3" t="n">
+        <v>12.11</v>
+      </c>
+      <c r="K10" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -2580,7 +2696,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="G11" s="3" t="n">
+        <v>32904</v>
+      </c>
+      <c r="H11" s="3" t="n">
+        <v>2851</v>
+      </c>
+      <c r="I11" s="3" t="n">
+        <v>35755</v>
+      </c>
+      <c r="J11" s="3" t="n">
+        <v>15.2</v>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -2615,7 +2743,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="G12" s="3" t="inlineStr">
+      <c r="G12" s="3" t="n">
+        <v>32997</v>
+      </c>
+      <c r="H12" s="3" t="n">
+        <v>3561</v>
+      </c>
+      <c r="I12" s="3" t="n">
+        <v>36558</v>
+      </c>
+      <c r="J12" s="3" t="n">
+        <v>17.06</v>
+      </c>
+      <c r="K12" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -2650,6 +2790,26 @@
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
           <t>N/A - fixture not yet implemented</t>
         </is>
       </c>
@@ -2683,6 +2843,26 @@
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="inlineStr">
+        <is>
           <t>N/A - fixture not yet implemented</t>
         </is>
       </c>
@@ -2716,7 +2896,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="G15" s="3" t="inlineStr">
+      <c r="G15" s="3" t="n">
+        <v>43838</v>
+      </c>
+      <c r="H15" s="3" t="n">
+        <v>13823</v>
+      </c>
+      <c r="I15" s="3" t="n">
+        <v>57661</v>
+      </c>
+      <c r="J15" s="3" t="n">
+        <v>52.37</v>
+      </c>
+      <c r="K15" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -2751,7 +2943,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="G16" s="3" t="inlineStr">
+      <c r="G16" s="3" t="n">
+        <v>21206</v>
+      </c>
+      <c r="H16" s="3" t="n">
+        <v>466</v>
+      </c>
+      <c r="I16" s="3" t="n">
+        <v>21672</v>
+      </c>
+      <c r="J16" s="3" t="n">
+        <v>3.73</v>
+      </c>
+      <c r="K16" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -2786,6 +2990,26 @@
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K17" s="3" t="inlineStr">
+        <is>
           <t>N/A - fixture not yet implemented</t>
         </is>
       </c>
@@ -2819,7 +3043,19 @@
           <t>FAIL</t>
         </is>
       </c>
-      <c r="G18" s="3" t="inlineStr">
+      <c r="G18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" s="3" t="n">
+        <v>240.03</v>
+      </c>
+      <c r="K18" s="3" t="inlineStr">
         <is>
           <t>Delegation stall / shortcut (deep-workflow non-termination, unresolved)</t>
         </is>
@@ -2854,7 +3090,19 @@
           <t>FAIL</t>
         </is>
       </c>
-      <c r="G19" s="3" t="inlineStr">
+      <c r="G19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" s="3" t="n">
+        <v>240.04</v>
+      </c>
+      <c r="K19" s="3" t="inlineStr">
         <is>
           <t>Delegation stall / shortcut (deep-workflow non-termination, unresolved)</t>
         </is>
@@ -2889,7 +3137,19 @@
           <t>FAIL</t>
         </is>
       </c>
-      <c r="G20" s="3" t="inlineStr">
+      <c r="G20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J20" s="3" t="n">
+        <v>240.04</v>
+      </c>
+      <c r="K20" s="3" t="inlineStr">
         <is>
           <t>Delegation stall / shortcut (deep-workflow non-termination, unresolved)</t>
         </is>
@@ -2924,7 +3184,19 @@
           <t>FAIL</t>
         </is>
       </c>
-      <c r="G21" s="3" t="inlineStr">
+      <c r="G21" s="3" t="n">
+        <v>32475</v>
+      </c>
+      <c r="H21" s="3" t="n">
+        <v>8724</v>
+      </c>
+      <c r="I21" s="3" t="n">
+        <v>41199</v>
+      </c>
+      <c r="J21" s="3" t="n">
+        <v>50.45</v>
+      </c>
+      <c r="K21" s="3" t="inlineStr">
         <is>
           <t>Premature mutation proposal (not yet fixed)</t>
         </is>
@@ -2959,6 +3231,26 @@
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I22" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K22" s="3" t="inlineStr">
+        <is>
           <t>N/A - fixture not yet implemented</t>
         </is>
       </c>
@@ -2992,7 +3284,19 @@
           <t>FAIL</t>
         </is>
       </c>
-      <c r="G23" s="3" t="inlineStr">
+      <c r="G23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J23" s="3" t="n">
+        <v>240.01</v>
+      </c>
+      <c r="K23" s="3" t="inlineStr">
         <is>
           <t>Delegation stall / shortcut (deep-workflow non-termination, unresolved)</t>
         </is>
@@ -3027,7 +3331,19 @@
           <t>FAIL</t>
         </is>
       </c>
-      <c r="G24" s="3" t="inlineStr">
+      <c r="G24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24" s="3" t="n">
+        <v>240.01</v>
+      </c>
+      <c r="K24" s="3" t="inlineStr">
         <is>
           <t>Delegation stall / shortcut (deep-workflow non-termination, unresolved)</t>
         </is>
@@ -3062,7 +3378,19 @@
           <t>FAIL</t>
         </is>
       </c>
-      <c r="G25" s="3" t="inlineStr">
+      <c r="G25" s="3" t="n">
+        <v>105286</v>
+      </c>
+      <c r="H25" s="3" t="n">
+        <v>20774</v>
+      </c>
+      <c r="I25" s="3" t="n">
+        <v>126060</v>
+      </c>
+      <c r="J25" s="3" t="n">
+        <v>221.46</v>
+      </c>
+      <c r="K25" s="3" t="inlineStr">
         <is>
           <t>Delegation stall / shortcut (deep-workflow non-termination, unresolved)</t>
         </is>
@@ -3097,7 +3425,19 @@
           <t>FAIL</t>
         </is>
       </c>
-      <c r="G26" s="3" t="inlineStr">
+      <c r="G26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J26" s="3" t="n">
+        <v>90.02</v>
+      </c>
+      <c r="K26" s="3" t="inlineStr">
         <is>
           <t>Provider/model latency instability</t>
         </is>
@@ -3132,7 +3472,19 @@
           <t>FAIL</t>
         </is>
       </c>
-      <c r="G27" s="3" t="inlineStr">
+      <c r="G27" s="3" t="n">
+        <v>10590</v>
+      </c>
+      <c r="H27" s="3" t="n">
+        <v>8192</v>
+      </c>
+      <c r="I27" s="3" t="n">
+        <v>18782</v>
+      </c>
+      <c r="J27" s="3" t="n">
+        <v>40.3</v>
+      </c>
+      <c r="K27" s="3" t="inlineStr">
         <is>
           <t>Provider/model latency instability</t>
         </is>
@@ -3167,7 +3519,19 @@
           <t>FAIL</t>
         </is>
       </c>
-      <c r="G28" s="3" t="inlineStr">
+      <c r="G28" s="3" t="n">
+        <v>43562</v>
+      </c>
+      <c r="H28" s="3" t="n">
+        <v>9830</v>
+      </c>
+      <c r="I28" s="3" t="n">
+        <v>53392</v>
+      </c>
+      <c r="J28" s="3" t="n">
+        <v>39.05</v>
+      </c>
+      <c r="K28" s="3" t="inlineStr">
         <is>
           <t>Provider/model latency instability</t>
         </is>
@@ -3202,7 +3566,19 @@
           <t>FAIL</t>
         </is>
       </c>
-      <c r="G29" s="3" t="inlineStr">
+      <c r="G29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J29" s="3" t="n">
+        <v>60.03</v>
+      </c>
+      <c r="K29" s="3" t="inlineStr">
         <is>
           <t>Not yet triaged</t>
         </is>
@@ -3237,7 +3613,19 @@
           <t>FAIL</t>
         </is>
       </c>
-      <c r="G30" s="3" t="inlineStr">
+      <c r="G30" s="3" t="n">
+        <v>60048</v>
+      </c>
+      <c r="H30" s="3" t="n">
+        <v>6148</v>
+      </c>
+      <c r="I30" s="3" t="n">
+        <v>66196</v>
+      </c>
+      <c r="J30" s="3" t="n">
+        <v>41.39</v>
+      </c>
+      <c r="K30" s="3" t="inlineStr">
         <is>
           <t>Not yet triaged (partial completion - artifact-write timing)</t>
         </is>
@@ -3272,7 +3660,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="G31" s="3" t="inlineStr">
+      <c r="G31" s="3" t="n">
+        <v>21548</v>
+      </c>
+      <c r="H31" s="3" t="n">
+        <v>2695</v>
+      </c>
+      <c r="I31" s="3" t="n">
+        <v>24243</v>
+      </c>
+      <c r="J31" s="3" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="K31" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -3307,7 +3707,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="G32" s="3" t="inlineStr">
+      <c r="G32" s="3" t="n">
+        <v>32488</v>
+      </c>
+      <c r="H32" s="3" t="n">
+        <v>2897</v>
+      </c>
+      <c r="I32" s="3" t="n">
+        <v>35385</v>
+      </c>
+      <c r="J32" s="3" t="n">
+        <v>12.18</v>
+      </c>
+      <c r="K32" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -3342,7 +3754,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="G33" s="3" t="inlineStr">
+      <c r="G33" s="3" t="n">
+        <v>21544</v>
+      </c>
+      <c r="H33" s="3" t="n">
+        <v>1732</v>
+      </c>
+      <c r="I33" s="3" t="n">
+        <v>23276</v>
+      </c>
+      <c r="J33" s="3" t="n">
+        <v>8.039999999999999</v>
+      </c>
+      <c r="K33" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -3377,7 +3801,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="G34" s="3" t="inlineStr">
+      <c r="G34" s="3" t="n">
+        <v>44221</v>
+      </c>
+      <c r="H34" s="3" t="n">
+        <v>4790</v>
+      </c>
+      <c r="I34" s="3" t="n">
+        <v>49011</v>
+      </c>
+      <c r="J34" s="3" t="n">
+        <v>21.97</v>
+      </c>
+      <c r="K34" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -3412,7 +3848,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="G35" s="3" t="inlineStr">
+      <c r="G35" s="3" t="n">
+        <v>44123</v>
+      </c>
+      <c r="H35" s="3" t="n">
+        <v>7760</v>
+      </c>
+      <c r="I35" s="3" t="n">
+        <v>51883</v>
+      </c>
+      <c r="J35" s="3" t="n">
+        <v>30.29</v>
+      </c>
+      <c r="K35" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -3447,7 +3895,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="G36" s="3" t="inlineStr">
+      <c r="G36" s="3" t="n">
+        <v>44312</v>
+      </c>
+      <c r="H36" s="3" t="n">
+        <v>5559</v>
+      </c>
+      <c r="I36" s="3" t="n">
+        <v>49871</v>
+      </c>
+      <c r="J36" s="3" t="n">
+        <v>20.99</v>
+      </c>
+      <c r="K36" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -3482,7 +3942,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="G37" s="3" t="inlineStr">
+      <c r="G37" s="3" t="n">
+        <v>32814</v>
+      </c>
+      <c r="H37" s="3" t="n">
+        <v>3228</v>
+      </c>
+      <c r="I37" s="3" t="n">
+        <v>36042</v>
+      </c>
+      <c r="J37" s="3" t="n">
+        <v>13.35</v>
+      </c>
+      <c r="K37" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -3517,7 +3989,19 @@
           <t>FAIL</t>
         </is>
       </c>
-      <c r="G38" s="3" t="inlineStr">
+      <c r="G38" s="3" t="n">
+        <v>66945</v>
+      </c>
+      <c r="H38" s="3" t="n">
+        <v>11366</v>
+      </c>
+      <c r="I38" s="3" t="n">
+        <v>78311</v>
+      </c>
+      <c r="J38" s="3" t="n">
+        <v>41.37</v>
+      </c>
+      <c r="K38" s="3" t="inlineStr">
         <is>
           <t>Rule over-generalization / regression (open follow-up)</t>
         </is>
@@ -3552,7 +4036,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="G39" s="3" t="inlineStr">
+      <c r="G39" s="3" t="n">
+        <v>42641</v>
+      </c>
+      <c r="H39" s="3" t="n">
+        <v>3379</v>
+      </c>
+      <c r="I39" s="3" t="n">
+        <v>46020</v>
+      </c>
+      <c r="J39" s="3" t="n">
+        <v>14.61</v>
+      </c>
+      <c r="K39" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -3587,7 +4083,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="G40" s="3" t="inlineStr">
+      <c r="G40" s="3" t="n">
+        <v>21278</v>
+      </c>
+      <c r="H40" s="3" t="n">
+        <v>1057</v>
+      </c>
+      <c r="I40" s="3" t="n">
+        <v>22335</v>
+      </c>
+      <c r="J40" s="3" t="n">
+        <v>5.51</v>
+      </c>
+      <c r="K40" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -3622,17 +4130,35 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="G41" s="3" t="inlineStr">
+      <c r="G41" s="3" t="n">
+        <v>32812</v>
+      </c>
+      <c r="H41" s="3" t="n">
+        <v>4560</v>
+      </c>
+      <c r="I41" s="3" t="n">
+        <v>37372</v>
+      </c>
+      <c r="J41" s="3" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="K41" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
     </row>
-    <row r="42"/>
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
           <t>Live: 17/33 strict pass (52%). Routing-only pass: 20/33 (61%). 5 rows still pending_fixture.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Cost: 1,053,653 total tokens across 33 live runs (avg 31,929/run - undercounts delegated-subagent token use, see run_baseline_eval.py run_case docstring). Total latency: 2,198s across 33 runs. Most expensive single runs: hero-weekly-candidates (run 3): 126,060 tokens, reassign-parent-only (run 1): 78,311 tokens, family-outing-weekend (run 1): 66,196 tokens.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Cost Comparison sheet: before/after tokens and latency
step1-4_summary.xlsx: new Cost Comparison sheet matches the 20 cases
present in both the original pre-triage baseline and the current final
baseline, showing per-case token/latency deltas plus an explanation of
why tokens rose overall (previously-failing cases recorded 0 tokens
because they timed out before doing any real work) while latency fell
overall (fewer full-timeout rides).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/evaluations/step1-4_summary.xlsx
+++ b/evaluations/step1-4_summary.xlsx
@@ -13,6 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Step 4 - Prompt Changes" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Full Results" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regression Tests" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cost Comparison" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4450,4 +4451,884 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Cost Comparison - the 20 cases present in both the original 2026-09-04 pre-triage baseline and the current final baseline (results_baseline.csv), matched by case_id. Values are per-case averages across repeat runs, not sums, so cases with different repeat counts (1x then, up to 3x now) compare fairly. The 10 cases added later (to reach the 30-case dataset) have no 'before' state and are excluded from this comparison - see Full Results for their standalone numbers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>case_id</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>before_tokens</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>after_tokens</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>tokens_change</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>before_latency_s</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>after_latency_s</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>latency_change</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>before_pass</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>after_pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>approval-rejected</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>34640</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>57661</v>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>+66%</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>109.5</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>52.4</v>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>-52%</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>create-future-event</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>32858</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>35047</v>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>+7%</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>32.1</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>-15%</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>create-future-event-with-location</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>32785</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>35385</v>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>+8%</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>29.8</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>12.2</v>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>-59%</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>draft-both-parent-reminder</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>34676</v>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>36558</v>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>+5%</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>44.6</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>17.1</v>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>-62%</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>family-outing-weekend</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>66196</v>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>N/A (was 0 - failed/timed out before completing any work)</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>91.7</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>41.4</v>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>-55%</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>hero-weekly-candidates</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>42020</v>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>N/A (was 0 - failed/timed out before completing any work)</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>156.2</v>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>233.8</v>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>+50%</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>list-child-events</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>20947</v>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>22401</v>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>+7%</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>15.2</v>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>-21%</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>list-family-next-week</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>22518</v>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>23276</v>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>+3%</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>31.4</v>
+      </c>
+      <c r="F11" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>-74%</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>list-reminder-drafts</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>32831</v>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>36042</v>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>+10%</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>27.9</v>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>-52%</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>reject-past-event</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>33945</v>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>36971</v>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>+9%</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="F13" s="3" t="n">
+        <v>45.3</v>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>-0%</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>restore-event</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>33555</v>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>35755</v>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>+7%</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>34.3</v>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>15.2</v>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>-56%</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>same-child-conflict</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>N/A (both 0 - timed out both times)</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>60</v>
+      </c>
+      <c r="F15" s="3" t="n">
+        <v>60</v>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>+0%</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>same-parent-conflict</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>11365</v>
+      </c>
+      <c r="C16" s="3" t="n">
+        <v>13252</v>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>+17%</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>17.3</v>
+      </c>
+      <c r="F16" s="3" t="n">
+        <v>13.9</v>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>-20%</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>school-event-overlap</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>33537</v>
+      </c>
+      <c r="C17" s="3" t="n">
+        <v>41199</v>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>+23%</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>35.6</v>
+      </c>
+      <c r="F17" s="3" t="n">
+        <v>50.5</v>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>+42%</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>soft-delete-event</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>32181</v>
+      </c>
+      <c r="C18" s="3" t="n">
+        <v>34958</v>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>+9%</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>19.6</v>
+      </c>
+      <c r="F18" s="3" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>-38%</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>stale-weekly-option</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>N/A (both 0 - timed out both times)</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="n">
+        <v>60</v>
+      </c>
+      <c r="F19" s="3" t="n">
+        <v>60</v>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>+0%</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>untrusted-event-title-injection</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>22643</v>
+      </c>
+      <c r="C20" s="3" t="n">
+        <v>24243</v>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>+7%</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="F20" s="3" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>-65%</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>update-event-success</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="3" t="n">
+        <v>50255</v>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>N/A (was 0 - failed/timed out before completing any work)</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="n">
+        <v>60</v>
+      </c>
+      <c r="F21" s="3" t="n">
+        <v>24.4</v>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>-59%</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>vikram-availability-rule</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>11793</v>
+      </c>
+      <c r="C22" s="3" t="n">
+        <v>24058</v>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>+104%</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="n">
+        <v>21.1</v>
+      </c>
+      <c r="F22" s="3" t="n">
+        <v>56.5</v>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>+168%</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="I22" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>weekly-deep-planning</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>N/A (both 0 - timed out both times)</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="n">
+        <v>194.8</v>
+      </c>
+      <c r="F23" s="3" t="n">
+        <v>240</v>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>+23%</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>AGGREGATE (sum of per-case averages, 20 matched cases): tokens 390,274 -&gt; 615,277 (+58%). Latency 1,116s -&gt; 1,006s (-10%).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Why tokens went UP overall despite fixes: several previously-broken cases (approval-rejected, vikram-availability-rule, update-event-success, hero-weekly-candidates, family-outing-weekend) recorded 0 or near-0 tokens before because they timed out or failed before completing any real reasoning - a token count of 0 there means 'did no useful work,' not 'was cheap.' After the fixes, those same cases now do the actual required tool calls and reasoning, which costs real tokens. The token increase is mostly the cost of doing the work correctly, not inefficiency.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Why latency went DOWN overall despite that: fewer cases now ride out a full 60s/240s timeout ceiling with nothing to show for it - e.g. update-event-success dropped from 60.0s (always timed out) to 24.4s (now completes quickly and correctly). The exception is vikram-availability-rule (+168% latency) and weekly-deep-planning (+23%), which now do more required work per attempt (or consistently hit the full ceiling instead of sometimes crashing early via a provider timeout) - see WEEK4_HANDOVER_2026-09-04.md for the full explanation of each.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>